<commit_message>
Add Frontend, Upload UI, and Admin Auth
</commit_message>
<xml_diff>
--- a/data/questions.xlsx
+++ b/data/questions.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2034,6 +2034,426 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Q0038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Can you walk us through a product you launched that required navigating complex regulatory requirements in financial services?</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Product Manager - FinTech Industry</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Role Relevance</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Specific product details, awareness of compliance constraints, how they collaborated with legal/compliance, and the outcome.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>vague answer about compliance</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Q0039</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>How do you prioritize features when you have competing demands from engineering, design, and business stakeholders?</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Product Manager - FinTech Industry</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Problem Solving</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Situational</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Use of prioritization frameworks (e.g., RICE, MoSCoW), how they handle conflict, data-driven decision making.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>no framework mentioned</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Q0040</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Describe a situation where user research changed your product direction significantly.</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Product Manager - FinTech Industry</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Communication Skills</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Research methods used, how insights were gathered, and how they influenced product decisions.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>no specific research method mentioned</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Q0041</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>How do you define and track the success of a new financial product after launch?</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Product Manager - FinTech Industry</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Role Relevance</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Profile-Grounded</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>KPIs mentioned (retention, activation, NPS, revenue), use of analytics tools, iterative approach.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>no KPIs given</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Q0042</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Tell me about a time you had to say no to a feature request from a key stakeholder. How did you handle it?</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Product Manager - FinTech Industry</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Leadership</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Confidence in decision-making, ability to communicate trade-offs, maintaining stakeholder relationships.</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>no mention of stakeholder communication</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Q0043</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>How do you stay current with FinTech trends and integrate emerging technologies like AI or blockchain into your product roadmap?</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Product Manager - FinTech Industry</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Training Development</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Profile-Grounded</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Specific technologies mentioned, sources of industry learning, real examples of integrating new tech.</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>vague answer about staying updated</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Q0044</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Describe a time when a product launch did not go as planned. What was your response?</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Product Manager - FinTech Industry</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Problem Solving</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Ownership of failure, corrective actions taken, lessons learned, speed of response.</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>blame shifted to team or external factors</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Q0045</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>How do you manage your product backlog and ensure the team is always working on the highest-value items?</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Product Manager - FinTech Industry</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Project Management</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Situational</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Tools used (Jira, Asana), grooming cadence, how value is assessed, collaboration with engineering.</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>no tools or process mentioned</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Q0046</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Can you describe your experience working with cross-functional teams including engineering, marketing, and compliance in a FinTech environment?</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Product Manager - FinTech Industry</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Communication Skills</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Profile-Grounded</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Examples of cross-functional collaboration, handling disagreements, ensuring alignment.</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>vague answer about teamwork</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Q0047</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>What strategies do you use to gather and incorporate customer feedback into an iterative product development cycle?</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Product Manager - FinTech Industry</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Role Relevance</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Situational</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Feedback channels (surveys, interviews, NPS), frequency of collection, how it feeds into roadmap decisions.</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>no specific feedback method mentioned</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>